<commit_message>
Clean up Step 1 sample workbook formatting
</commit_message>
<xml_diff>
--- a/public/samples/Combined - EXAMINATION TIMETABLE - Input.xlsx
+++ b/public/samples/Combined - EXAMINATION TIMETABLE - Input.xlsx
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W68"/>
+  <dimension ref="A1:O68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="1"/>
   <cols>
     <col width="10.77734375" customWidth="1" style="9" min="1" max="1"/>
@@ -881,30 +881,6 @@
       <c r="O5" s="19" t="n">
         <v>0.5034722222222222</v>
       </c>
-      <c r="P5" s="7" t="n"/>
-      <c r="Q5" s="7" t="n"/>
-      <c r="R5" s="7" t="n"/>
-      <c r="S5" s="7" t="inlineStr">
-        <is>
-          <t>27/10/2025</t>
-        </is>
-      </c>
-      <c r="T5" s="7" t="inlineStr">
-        <is>
-          <t>8655/01</t>
-        </is>
-      </c>
-      <c r="U5" s="7" t="inlineStr">
-        <is>
-          <t>AM</t>
-        </is>
-      </c>
-      <c r="V5" s="7" t="n">
-        <v>180</v>
-      </c>
-      <c r="W5" s="7" t="n">
-        <v>225</v>
-      </c>
     </row>
     <row r="6" outlineLevel="1" s="9">
       <c r="A6" s="2" t="inlineStr">

</xml_diff>